<commit_message>
Retire method guides, demo repo, and stale templates paths
Items 18, 19, 20, 22; D4.

- Delete the five course-invariant method guides (Kumu owns method) and
  merge the VAS/IFRS/GAAP quickref into the Performance Ratios
  gaap-conversion-quickref; guides/ is now empty and gone.
- Delete demo-portfolio-repo/; templates/portfolio/firstname-lastname/
  is the one sample.
- Stage-brief template: capabilities/, no local path or draft status,
  dead memo and README paths repaired. templates README index matches
  the files; prompt-log line fixed; employer claims removed. Portfolio
  repo name is firstname-lastname throughout; the bio is drafted by
  the student and AI reviews only.
- Ratios workbook Cover: two dead paths repointed (shared strings only).
- FIN-321 summer-2026: past-term banner, lms-docx/ removed, two dead
  canonical stage links repointed.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/spreadsheets/performance-ratios-template.xlsx
+++ b/templates/spreadsheets/performance-ratios-template.xlsx
@@ -741,13 +741,13 @@
     <t>See:</t>
   </si>
   <si>
-    <t>docs/templates/spec-template.md (repo-level)</t>
+    <t>templates/spec-template.md (repo-level)</t>
   </si>
   <si>
     <t>Course:</t>
   </si>
   <si>
-    <t>courses/BUS-629-VEMBA-International-Corporate-Finance/</t>
+    <t>courses/International-Corporate-Finance/</t>
   </si>
   <si>
     <t>Prepared per UH Mānoa brand standards (docs/_branding/design.json). Primary green #024731 · Open Sans typography · ADA-compliant contrast.</t>

</xml_diff>

<commit_message>
Clear post-wave leftovers: email asks, branding, markup, legend
After-the-wave leftovers from the three-surfaces review: IC Stage 2
markup as a question; BUS-313 grades defer to grading-scale.md; every
student-facing @hawaii.edu ask replaced (Adam 2026-10-05, no UH Claude
license); branding binaries to #024731 with an instructor footer;
workbook Cover named-range text fixed; sample AGENTS.md legend matches
the house standard. DIG-15.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/spreadsheets/performance-ratios-template.xlsx
+++ b/templates/spreadsheets/performance-ratios-template.xlsx
@@ -687,10 +687,10 @@
     <t>Prefix / Pattern</t>
   </si>
   <si>
-    <t>BAL_[item]_[yr]</t>
-  </si>
-  <si>
-    <t>Balance-sheet line items, suffixed with fiscal year (e.g., BAL_assets_total_2024).</t>
+    <t>BAL_[item]_curr, BAL_[item]_prior</t>
+  </si>
+  <si>
+    <t>Balance-sheet line items, suffixed _curr for the current year or _prior for the prior year (e.g., BAL_assets_total_curr).</t>
   </si>
   <si>
     <t>INC_[item]</t>

</xml_diff>